<commit_message>
Configurado Excel com formato específico - atividades detalhadas e layout conforme imagem
</commit_message>
<xml_diff>
--- a/teste_trilha_controle.xlsx
+++ b/teste_trilha_controle.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="32">
   <si>
     <t>Atividade</t>
   </si>
@@ -31,52 +31,85 @@
     <t>Observações</t>
   </si>
   <si>
-    <t>1. Análise inicial da trilha</t>
-  </si>
-  <si>
-    <t>2. Execução das atividades principais</t>
-  </si>
-  <si>
-    <t>3. Validação e testes</t>
-  </si>
-  <si>
-    <t>4. Finalização e documentação</t>
-  </si>
-  <si>
-    <t>A definir</t>
-  </si>
-  <si>
-    <t>Análise</t>
-  </si>
-  <si>
-    <t>Execução</t>
-  </si>
-  <si>
-    <t>Validação</t>
-  </si>
-  <si>
-    <t>Finalização</t>
-  </si>
-  <si>
-    <t>Não</t>
-  </si>
-  <si>
-    <t>Primeira etapa da trilha</t>
-  </si>
-  <si>
-    <t>Atividades específicas da trilha</t>
-  </si>
-  <si>
-    <t>Verificação dos resultados</t>
-  </si>
-  <si>
-    <t>Conclusão da trilha</t>
+    <t>CMR205.2 - BPH004251 - 1. Relatório de estoques / Disponibilidade do Produto</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH004047 - 2. Criar contrato de compra</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003890 - 3. Aprovar contrato de Compras</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003890 - 4. Consultar aprovação de workflow</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003625 - 5. Avaliar fluxo de caixa diário</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH004065 - 6. Criar pedido de compra vinculado ao contrato</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003386 - 7. Realizar Pré Validação Fiscal do Pedido de Compra [VALIDAÇÃO]</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003625 - 8. Avaliar fluxo de caixa diário</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH004054 - 9. Lançar contrato de Venda</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH004301 - 10. Aprovar contrato de Venda</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003625 - 11. Avaliar fluxo de caixa diário</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH004055 - 12. Lançar ordem de venda no sistema</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH003523 - 13. Realizar Pré Validação Fiscal da Ordem de Venda [VALIDAÇÃO]</t>
+  </si>
+  <si>
+    <t>CMR205.2 - BPH001162 - 14. Identificar a demanda na plataforma</t>
+  </si>
+  <si>
+    <t>bruno.lobo@sipal.com.br</t>
+  </si>
+  <si>
+    <t>lucas.sbardella@sipal.com.br</t>
+  </si>
+  <si>
+    <t>caroline.silva@sipal.com.br</t>
+  </si>
+  <si>
+    <t>everton.siqueira@sipal.com.br</t>
+  </si>
+  <si>
+    <t>anna.santos@sipal.com.br</t>
+  </si>
+  <si>
+    <t>luiz.ferreira@sipal.com.br</t>
+  </si>
+  <si>
+    <t>simone.tessaro@sipal.com.br</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>Tarken</t>
   </si>
   <si>
     <t>CMR205.2 - CMR205.2 - SD Fertilizantes - Compra Direta + Venda com Troca De Notas</t>
   </si>
   <si>
-    <t>Gerado em: 28/07/2025 17:42:35</t>
+    <t>CMR205.2 - SD Fertilizantes - Compra Direta + Venda com Troca De Notas - Ori. Fabrica / Dest. Cliente - (Compra FOB e Venda CIF - À Prazo) V - [C3]</t>
+  </si>
+  <si>
+    <t>Massa de dados não informada</t>
+  </si>
+  <si>
+    <t>Gerado em: 28/07/2025 17:52:18</t>
   </si>
 </sst>
 </file>
@@ -454,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="60.7109375" customWidth="1"/>
@@ -465,98 +498,222 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>17</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="B11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="B15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="B16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
+      <c r="B20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>